<commit_message>
Fix Cr/Li10Ge relax records and add RMSD-vs-expert comparison
relax.xlsx: Cr and Li10Ge(PS6)2 had converged (rx_ runs, returncode 0)
but were recorded as failed; fill their E0 in the vaspagent row and
sources sheet and bump the vaspagent success rate to 1.0. Cr is annotated
because the agent input is Cr35 (35 atoms) while the ground truth is Cr2
(2 atoms), so totals are compared per-atom (-9.41 vs -9.50 eV/atom).

relax_new.xlsx: StructureMatcher RMSD (normalized) of 5 groups (4 workflow
models + agent) against the expert relaxed structures, with per-group
n_matched / mean / median summary.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/relax.xlsx
+++ b/relax.xlsx
@@ -125,6 +125,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>accuracy-check</author>
+  </authors>
+  <commentList>
+    <comment ref="M8" authorId="0" shapeId="0">
+      <text>
+        <t>Cr: agent input data/relax/Cr is Cr35 (35 atoms, E0=-329.38014). ground truth row is Cr2 (2 atoms, -19.009246). Totals NOT directly comparable; compare per-atom: agent -9.4109 vs GT -9.5046 eV/atom (Δ0.094).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1510,10 +1525,8 @@
       <c r="L8" t="n">
         <v>-152.38851</v>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
+      <c r="M8" t="n">
+        <v>-329.38014</v>
       </c>
       <c r="N8" t="n">
         <v>-96.208468</v>
@@ -1536,10 +1549,8 @@
       <c r="T8" t="n">
         <v>-683.00951</v>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
+      <c r="U8" t="n">
+        <v>-210.69189</v>
       </c>
       <c r="V8" t="n">
         <v>-193.24805</v>
@@ -1605,11 +1616,12 @@
         <v>-16.439068</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2948,7 +2960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2978,6 +2990,11 @@
           <t>candidate_count</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3165,14 +3182,21 @@
           <t>Cr</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="B12" t="n">
+        <v>-329.38014</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>runs/rx_Cr</t>
+        </is>
+      </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Cr35 (35 atoms); GT is Cr2 (2 atoms) -&gt; compare per-atom (agent -9.4109 vs GT -9.5046 eV/atom). Converged (returncode 0).</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -3253,14 +3277,21 @@
           <t>Li10Ge(PS6)2</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="B17" t="n">
+        <v>-210.69189</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>runs/rx_Li10Ge(PS6)2</t>
+        </is>
+      </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>49-atom cell, same as GT. Converged; matches GT (Δ0.076 eV).</t>
+        </is>
       </c>
     </row>
     <row r="18">

</xml_diff>